<commit_message>
Security audit: npm audit and pip-audit to 0 (upgrades; python-jose replaced by PyJWT); SECRET_KEY length warning
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="399">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1135,7 +1135,13 @@
     <t xml:space="preserve">No high or critical issues left unexplained</t>
   </si>
   <si>
-    <t xml:space="preserve">Tool (step 3)</t>
+    <t xml:space="preserve">Tool: npm audit + pip-audit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/security/: npm_audit_2026-10-22_before/after.txt, pip_audit_2026-10-22_before/after.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before: frontend 3 high, backend 58 advisories in 6 packages. After: 0 and 0 (upgrades; python-jose replaced by PyJWT). 140 pytest + 13 browser tests pass after the changes</t>
   </si>
   <si>
     <t xml:space="preserve">TC-66</t>
@@ -4054,17 +4060,23 @@
       <c r="G66" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="H66" s="3"/>
-      <c r="I66" s="3"/>
+      <c r="H66" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="I66" s="3" t="s">
+        <v>371</v>
+      </c>
       <c r="J66" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="K66" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="K66" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="L66" s="3"/>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>365</v>
@@ -4073,16 +4085,16 @@
         <v>208</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="H67" s="3"/>
       <c r="I67" s="3"/>
@@ -4094,7 +4106,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>365</v>
@@ -4103,16 +4115,16 @@
         <v>208</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="H68" s="3"/>
       <c r="I68" s="3"/>
@@ -4163,12 +4175,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4176,13 +4188,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>163</v>
@@ -4429,7 +4441,7 @@
       </c>
       <c r="C16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A16,'Test cases'!$J$2:$J$68,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A16,'Test cases'!$J$2:$J$68,"Fail")</f>
@@ -4437,12 +4449,12 @@
       </c>
       <c r="E16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A16,'Test cases'!$J$2:$J$68,"Not run")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">SUM(B5:B16)</f>
@@ -4450,7 +4462,7 @@
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">SUM(C5:C16)</f>
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D17" s="8" t="n">
         <f aca="false">SUM(D5:D16)</f>
@@ -4458,7 +4470,7 @@
       </c>
       <c r="E17" s="8" t="n">
         <f aca="false">SUM(E5:E16)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4470,7 +4482,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -4479,7 +4491,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"1")</f>
@@ -4494,7 +4506,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"2")</f>
@@ -4509,7 +4521,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"3")</f>
@@ -4524,7 +4536,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"4")</f>
@@ -4568,42 +4580,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Accessibility: Lighthouse 100 on 4 pages, axe scan 0 problems on 18 pages (WCAG 2.2 AA), keyboard tests; 16 browser tests passed; TC-66 Pass
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="401">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1150,13 +1150,19 @@
     <t xml:space="preserve">Accessibility</t>
   </si>
   <si>
-    <t xml:space="preserve">Lighthouse on Dashboard, My Profile, Job Detail, Applicants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accessibility score recorded; serious issues fixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool (step 4)</t>
+    <t xml:space="preserve">Lighthouse (Chrome DevTools, desktop, Accessibility) on Sign in, Job Matches, Job Detail and View applicants; axe-core scan of 18 pages of all roles (incl. Dashboard, My Profile); Job Matches and View applicants with the keyboard only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No serious accessibility problems left; Lighthouse accessibility score recorded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Lighthouse + axe-core scan (Playwright) + keyboard tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/lighthouse/ (4 reports); docs/evidence/e2e/accessibility.json and accessibility_before_2026-10-22.md; Playwright 22 Oct (16 passed): 5-accessibility.spec.js</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lighthouse accessibility 100 on Sign in (93 before the fixes), Job Matches, Job Detail and View applicants (desktop). axe-core, WCAG 2.2 AA + best practice: 0 problems on 18 pages (before: low contrast on 17 pages, 2 unlabelled tick boxes, a colour-only link, small buttons, missing landmarks). Job and applicant lists open with Tab + Enter</t>
   </si>
   <si>
     <t xml:space="preserve">TC-67</t>
@@ -4096,17 +4102,23 @@
       <c r="G67" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="H67" s="3"/>
-      <c r="I67" s="3"/>
+      <c r="H67" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="I67" s="3" t="s">
+        <v>378</v>
+      </c>
       <c r="J67" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="K67" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="K67" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="L67" s="3"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>365</v>
@@ -4115,16 +4127,16 @@
         <v>208</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="H68" s="3"/>
       <c r="I68" s="3"/>
@@ -4175,12 +4187,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4188,13 +4200,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>163</v>
@@ -4441,7 +4453,7 @@
       </c>
       <c r="C16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A16,'Test cases'!$J$2:$J$68,"Pass")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A16,'Test cases'!$J$2:$J$68,"Fail")</f>
@@ -4449,12 +4461,12 @@
       </c>
       <c r="E16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A16,'Test cases'!$J$2:$J$68,"Not run")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">SUM(B5:B16)</f>
@@ -4462,7 +4474,7 @@
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">SUM(C5:C16)</f>
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D17" s="8" t="n">
         <f aca="false">SUM(D5:D16)</f>
@@ -4470,7 +4482,7 @@
       </c>
       <c r="E17" s="8" t="n">
         <f aca="false">SUM(E5:E16)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4482,7 +4494,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -4491,7 +4503,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"1")</f>
@@ -4506,7 +4518,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"2")</f>
@@ -4521,7 +4533,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"3")</f>
@@ -4536,7 +4548,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"4")</f>
@@ -4580,42 +4592,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lighthouse on all 33 pages (100 each); fix blank page on a malformed link; label every form field; 17 browser tests
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="402">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1150,7 +1150,7 @@
     <t xml:space="preserve">Accessibility</t>
   </si>
   <si>
-    <t xml:space="preserve">Lighthouse (Chrome DevTools, desktop, Accessibility) on Sign in, Job Matches, Job Detail and View applicants; axe-core scan of 18 pages of all roles (incl. Dashboard, My Profile); Job Matches and View applicants with the keyboard only</t>
+    <t xml:space="preserve">Lighthouse (desktop, Accessibility) on every page of every role: 4 by hand in Chrome DevTools, all 33 by frontend/scripts/lighthouse_all.mjs; axe-core scan of 33 pages, pop-ups and forms (5-accessibility.spec.js); Job Matches and View applicants with the keyboard only</t>
   </si>
   <si>
     <t xml:space="preserve">No serious accessibility problems left; Lighthouse accessibility score recorded</t>
@@ -1159,10 +1159,13 @@
     <t xml:space="preserve">Tool: Lighthouse + axe-core scan (Playwright) + keyboard tests</t>
   </si>
   <si>
-    <t xml:space="preserve">docs/evidence/lighthouse/ (4 reports); docs/evidence/e2e/accessibility.json and accessibility_before_2026-10-22.md; Playwright 22 Oct (16 passed): 5-accessibility.spec.js</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lighthouse accessibility 100 on Sign in (93 before the fixes), Job Matches, Job Detail and View applicants (desktop). axe-core, WCAG 2.2 AA + best practice: 0 problems on 18 pages (before: low contrast on 17 pages, 2 unlabelled tick boxes, a colour-only link, small buttons, missing landmarks). Job and applicant lists open with Tab + Enter</t>
+    <t xml:space="preserve">docs/evidence/lighthouse/ (4 by hand) and lighthouse/all/ (33 + summary.md); docs/evidence/e2e/accessibility.json and accessibility_before_2026-10-22.md; 5-accessibility.spec.js (17 passed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lighthouse accessibility 100 on 33 of 33 pages (Sign in was 93 before the fixes). axe-core, WCAG 2.2 AA + best practice: 0 problems on 33 pages and states (before: low contrast on 17 pages, unlabelled tick boxes and form fields, links shown by colour only, small buttons, missing landmarks). Job and applicant lists open with Tab + Enter. The all-pages run also found a crash on a malformed link (fixed, browser test added)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 Oct 2026</t>
   </si>
   <si>
     <t xml:space="preserve">TC-67</t>
@@ -4112,13 +4115,13 @@
         <v>21</v>
       </c>
       <c r="K67" s="3" t="s">
-        <v>22</v>
+        <v>379</v>
       </c>
       <c r="L67" s="3"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>365</v>
@@ -4127,16 +4130,16 @@
         <v>208</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="H68" s="3"/>
       <c r="I68" s="3"/>
@@ -4187,12 +4190,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4200,13 +4203,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>163</v>
@@ -4466,7 +4469,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">SUM(B5:B16)</f>
@@ -4494,7 +4497,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -4503,7 +4506,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"1")</f>
@@ -4518,7 +4521,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"2")</f>
@@ -4533,7 +4536,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"3")</f>
@@ -4548,7 +4551,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"4")</f>
@@ -4592,42 +4595,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Test cases: TC-68 other browsers (5 x 17 passed), TC-69 real MongoDB (4 passed); 65 of 69 Pass
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="418">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1181,6 +1181,54 @@
   </si>
   <si>
     <t xml:space="preserve">Tool (step 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Works in other browsers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run the 17 browser tests in Chromium, Google Chrome, Microsoft Edge, Firefox and WebKit (Safari's engine): frontend/scripts/all_browsers.sh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All tests pass in each browser; applying confirmed within 1 s (Google RAIL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Playwright E2E (5 browsers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/e2e/run_2026-10-23.txt and firefox/, webkit/, edge/, chrome/ (run logs, results, screenshots, accessibility scans)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 of 17 in every browser. Click to "Applied": Chromium 164 ms, Firefox 186 ms, WebKit 413 ms, Edge 163 ms, Chrome 159 ms. In WebKit the keyboard tests focus the link directly (WebKit, like Safari, leaves links out of Tab by default)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not tested on real Safari (no Mac); WebKit is its engine. Phones and tablets out of scope (designed for laptops)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MongoDB for real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With MongoDB running: python -m pytest tests/test_mongodb_real.py (a separate skillmap_test database)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indexes incl. the 18-month expiry exist; a chat is saved, listed, reopened, continued and deleted; another student can't reach it; Download my data and Delete my account cover MongoDB; an evaluation run is saved and read back</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automated (real MongoDB server)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest 23 Oct (176 passed): docs/evidence/tests/pytest_2026-10-23.txt, tests/test_mongodb_real.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As expected: 4 of 4 against the real server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skipped with a message when MongoDB is off; the other tests use stand-ins</t>
   </si>
   <si>
     <t xml:space="preserve">SkillMap system testing — summary</t>
@@ -1698,7 +1746,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -4149,6 +4197,82 @@
       <c r="K68" s="3"/>
       <c r="L68" s="3"/>
     </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="I69" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="J69" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K69" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="L69" s="3" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="I70" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="J70" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K70" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="L70" s="3" t="s">
+        <v>400</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L68"/>
   <conditionalFormatting sqref="J2:J68">
@@ -4160,7 +4284,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J68" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J70" type="list">
       <formula1>"Pass,Fail,Not run"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4190,12 +4314,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>385</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>386</v>
+        <v>402</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4203,13 +4327,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>387</v>
+        <v>403</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>163</v>
@@ -4220,19 +4344,19 @@
         <v>13</v>
       </c>
       <c r="B5" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A5)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A5)</f>
         <v>6</v>
       </c>
       <c r="C5" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A5,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A5,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>6</v>
       </c>
       <c r="D5" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A5,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A5,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E5" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A5,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A5,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>0</v>
       </c>
     </row>
@@ -4241,19 +4365,19 @@
         <v>53</v>
       </c>
       <c r="B6" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A6)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A6)</f>
         <v>4</v>
       </c>
       <c r="C6" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A6,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A6,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>4</v>
       </c>
       <c r="D6" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A6,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A6,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E6" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A6,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A6,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>0</v>
       </c>
     </row>
@@ -4262,19 +4386,19 @@
         <v>75</v>
       </c>
       <c r="B7" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A7)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A7)</f>
         <v>5</v>
       </c>
       <c r="C7" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A7,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A7,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>5</v>
       </c>
       <c r="D7" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A7,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A7,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E7" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A7,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A7,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>0</v>
       </c>
     </row>
@@ -4283,19 +4407,19 @@
         <v>103</v>
       </c>
       <c r="B8" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A8)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A8)</f>
         <v>6</v>
       </c>
       <c r="C8" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A8,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A8,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>6</v>
       </c>
       <c r="D8" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A8,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A8,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E8" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A8,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A8,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>0</v>
       </c>
     </row>
@@ -4304,19 +4428,19 @@
         <v>136</v>
       </c>
       <c r="B9" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A9)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A9)</f>
         <v>6</v>
       </c>
       <c r="C9" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A9,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A9,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>5</v>
       </c>
       <c r="D9" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A9,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A9,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E9" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A9,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A9,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>1</v>
       </c>
     </row>
@@ -4325,19 +4449,19 @@
         <v>170</v>
       </c>
       <c r="B10" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A10)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A10)</f>
         <v>7</v>
       </c>
       <c r="C10" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A10,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A10,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>7</v>
       </c>
       <c r="D10" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A10,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A10,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E10" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A10,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A10,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>0</v>
       </c>
     </row>
@@ -4346,19 +4470,19 @@
         <v>207</v>
       </c>
       <c r="B11" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A11)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A11)</f>
         <v>13</v>
       </c>
       <c r="C11" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A11,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A11,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>13</v>
       </c>
       <c r="D11" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A11,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A11,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E11" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A11,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A11,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>0</v>
       </c>
     </row>
@@ -4367,19 +4491,19 @@
         <v>274</v>
       </c>
       <c r="B12" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A12)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A12)</f>
         <v>3</v>
       </c>
       <c r="C12" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A12,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A12,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>3</v>
       </c>
       <c r="D12" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A12,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A12,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E12" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A12,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A12,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>0</v>
       </c>
     </row>
@@ -4388,19 +4512,19 @@
         <v>291</v>
       </c>
       <c r="B13" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A13)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A13)</f>
         <v>3</v>
       </c>
       <c r="C13" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A13,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A13,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>2</v>
       </c>
       <c r="D13" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A13,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A13,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E13" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A13,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A13,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>1</v>
       </c>
     </row>
@@ -4409,19 +4533,19 @@
         <v>307</v>
       </c>
       <c r="B14" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A14)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A14)</f>
         <v>6</v>
       </c>
       <c r="C14" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A14,'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A14,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>6</v>
       </c>
       <c r="D14" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A14,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A14,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E14" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A14,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A14,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>0</v>
       </c>
     </row>
@@ -4430,19 +4554,19 @@
         <v>339</v>
       </c>
       <c r="B15" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A15)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A15)</f>
+        <v>6</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A15,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>5</v>
       </c>
-      <c r="C15" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A15,'Test cases'!$J$2:$J$68,"Pass")</f>
-        <v>4</v>
-      </c>
       <c r="D15" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A15,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A15,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A15,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A15,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>1</v>
       </c>
     </row>
@@ -4451,33 +4575,33 @@
         <v>365</v>
       </c>
       <c r="B16" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$2:$B$68,A16)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$2:$B$70,A16)</f>
+        <v>4</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A16,'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>3</v>
       </c>
-      <c r="C16" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A16,'Test cases'!$J$2:$J$68,"Pass")</f>
-        <v>2</v>
-      </c>
       <c r="D16" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A16,'Test cases'!$J$2:$J$68,"Fail")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A16,'Test cases'!$J$2:$J$70,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E16" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$68,$A16,'Test cases'!$J$2:$J$68,"Not run")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$2:$B$70,$A16,'Test cases'!$J$2:$J$70,"Not run")</f>
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>387</v>
+        <v>403</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">SUM(B5:B16)</f>
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">SUM(C5:C16)</f>
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D17" s="8" t="n">
         <f aca="false">SUM(D5:D16)</f>
@@ -4497,7 +4621,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -4506,14 +4630,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>390</v>
+        <v>406</v>
       </c>
       <c r="B20" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"1")</f>
+        <f aca="false">COUNTIF('Test cases'!$C$2:$C$70,"1")</f>
         <v>10</v>
       </c>
       <c r="C20" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$C$2:$C$68,"1",'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$C$2:$C$70,"1",'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>10</v>
       </c>
       <c r="D20" s="7"/>
@@ -4521,14 +4645,14 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>391</v>
+        <v>407</v>
       </c>
       <c r="B21" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"2")</f>
+        <f aca="false">COUNTIF('Test cases'!$C$2:$C$70,"2")</f>
         <v>12</v>
       </c>
       <c r="C21" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$C$2:$C$68,"2",'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$C$2:$C$70,"2",'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>12</v>
       </c>
       <c r="D21" s="7"/>
@@ -4536,14 +4660,14 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>392</v>
+        <v>408</v>
       </c>
       <c r="B22" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"3")</f>
+        <f aca="false">COUNTIF('Test cases'!$C$2:$C$70,"3")</f>
         <v>6</v>
       </c>
       <c r="C22" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$C$2:$C$68,"3",'Test cases'!$J$2:$J$68,"Pass")</f>
+        <f aca="false">COUNTIFS('Test cases'!$C$2:$C$70,"3",'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>6</v>
       </c>
       <c r="D22" s="7"/>
@@ -4551,15 +4675,15 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>393</v>
+        <v>409</v>
       </c>
       <c r="B23" s="7" t="n">
-        <f aca="false">COUNTIF('Test cases'!$C$2:$C$68,"4")</f>
+        <f aca="false">COUNTIF('Test cases'!$C$2:$C$70,"4")</f>
+        <v>7</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$C$2:$C$70,"4",'Test cases'!$J$2:$J$70,"Pass")</f>
         <v>6</v>
-      </c>
-      <c r="C23" s="7" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$C$2:$C$68,"4",'Test cases'!$J$2:$J$68,"Pass")</f>
-        <v>5</v>
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="7"/>
@@ -4595,42 +4719,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>394</v>
+        <v>410</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>395</v>
+        <v>411</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>396</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>397</v>
+        <v>413</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>398</v>
+        <v>414</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>399</v>
+        <v>415</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>400</v>
+        <v>416</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>401</v>
+        <v>417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TC-53 forgot password tested by hand with real Gmail: Pass (evidence in docs/evidence/manual)
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -3606,16 +3606,24 @@
       </c>
       <c r="H54" s="14" t="inlineStr">
         <is>
-          <t>Needs the email settings</t>
-        </is>
-      </c>
-      <c r="I54" s="14" t="n"/>
+          <t>docs/evidence/manual/TC-53_1 to TC-53_7 (reset page, code email, code verified, password changed, old password refused, new password signs in)</t>
+        </is>
+      </c>
+      <c r="I54" s="14" t="inlineStr">
+        <is>
+          <t>Code arrived in Gmail within a minute, naming the account (tc53test), 15 minutes, single use. Code verified, new password set, "Password changed" message. Old password refused ("Invalid credentials", account not revealed); new password signs in. Real Gmail delivery (SMTP), test account weilinglow0926+tc53@gmail.com.</t>
+        </is>
+      </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="K54" s="14" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K54" s="14" t="inlineStr">
+        <is>
+          <t>24 Oct 2026</t>
+        </is>
+      </c>
       <c r="L54" s="14" t="n"/>
     </row>
     <row r="55" ht="23.25" customHeight="1" s="12">

</xml_diff>

<commit_message>
TC-53 forgot password tested by hand with real Gmail: Pass (8 screenshots in docs/evidence/manual)
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -3606,12 +3606,12 @@
       </c>
       <c r="H54" s="14" t="inlineStr">
         <is>
-          <t>docs/evidence/manual/TC-53_1 to TC-53_7 (reset page, code email, code verified, password changed, old password refused, new password signs in)</t>
+          <t>docs/evidence/manual/TC-53_1 to TC-53_8 (reset page, code email, code verified, password changed, old password refused, new password signs in, password-changed email)</t>
         </is>
       </c>
       <c r="I54" s="14" t="inlineStr">
         <is>
-          <t>Code arrived in Gmail within a minute, naming the account (tc53test), 15 minutes, single use. Code verified, new password set, "Password changed" message. Old password refused ("Invalid credentials", account not revealed); new password signs in. Real Gmail delivery (SMTP), test account weilinglow0926+tc53@gmail.com.</t>
+          <t>Code arrived in Gmail within a minute, naming the account (tc53test), 15 minutes, single use. Code verified, new password set, "Password changed" message. Old password refused ("Invalid credentials", account not revealed); new password signs in. A "password was changed" email followed, with the time and "other devices have been signed out". Real Gmail delivery (SMTP), test account weilinglow0926+tc53@gmail.com.</t>
         </is>
       </c>
       <c r="J54" s="14" t="inlineStr">

</xml_diff>

<commit_message>
TC-26 AI Assistant chat kept: Pass (4 screenshots); log how long each chat reply takes
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -2048,16 +2048,24 @@
       </c>
       <c r="H27" s="14" t="inlineStr">
         <is>
-          <t>Needs the Groq key and MongoDB</t>
-        </is>
-      </c>
-      <c r="I27" s="14" t="n"/>
+          <t>docs/evidence/manual/TC-26_1 to TC-26_4 (plan answered and listed, listed after signing in again, reopened, follow-up in the same chat)</t>
+        </is>
+      </c>
+      <c r="I27" s="14" t="inlineStr">
+        <is>
+          <t>Skill Development: "How do I start learning SQL joins?", 5 hours a week -&gt; learning plan (resources, 5-step table, portfolio project, Download plan). The chat was listed under Today; after leaving and signing in again it was still listed and reopened with the full plan; "And outer joins?" continued the same chat (one entry in the list). Real Groq + MongoDB. Note: the reply took noticeably long (being measured).</t>
+        </is>
+      </c>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="K27" s="14" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K27" s="14" t="inlineStr">
+        <is>
+          <t>24 Oct 2026</t>
+        </is>
+      </c>
       <c r="L27" s="14" t="n"/>
     </row>
     <row r="28" ht="34.5" customHeight="1" s="12">

</xml_diff>

<commit_message>
TC-64: Pass; Decide by in days (14/21/30/45); 'is live' banner counts graduates with all required skills; graduates who fit ranked by nice-to-have skills (research in references.md)
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -4256,16 +4256,24 @@
       </c>
       <c r="H65" s="14" t="inlineStr">
         <is>
-          <t>Stop the Groq key / network, then post</t>
-        </is>
-      </c>
-      <c r="I65" s="14" t="n"/>
+          <t>docs/evidence/manual/TC-64_1 (reader down: message and new heading), TC-64_2 (published with typed skills); backend/tests/test_extraction_records.py::test_reader_down_says_so_quickly_instead_of_no_skills</t>
+        </is>
+      </c>
+      <c r="I65" s="14" t="inlineStr">
+        <is>
+          <t>Backend started with a wrong GROQ_API_KEY. Read the skills: "SkillMap couldn't read the skills just now. Add them yourself below, or read the skills again in a few minutes" at the top of the skills, heading "Add the skills students are matched on". 3 required + 1 nice-to-have typed by hand; published and live. Found and fixed first (24 Oct): it used to wait 45 s and show no skills and no message; now about 9 s.</t>
+        </is>
+      </c>
       <c r="J65" s="14" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="K65" s="14" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K65" s="14" t="inlineStr">
+        <is>
+          <t>24 Oct 2026</t>
+        </is>
+      </c>
       <c r="L65" s="14" t="n"/>
     </row>
     <row r="66" ht="23.25" customHeight="1" s="12">

</xml_diff>

<commit_message>
Workbook: real-ad results in TC-18 and TC-20, new TC-75 to TC-78 (Ruff, Bandit, coverage, relation model); Bandit reasons on their own line
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Test cases'!$1:$1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Test cases'!$A$1:$L$75</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Test cases'!$A$1:$L$79</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="491">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -385,7 +385,16 @@
     <t xml:space="preserve">Pills for qualification, field, languages; no citizenship</t>
   </si>
   <si>
-    <t xml:space="preserve">pytest 21 Oct (137 passed): test_ad_requirements.py::test_live_job_requirements_read_by_the_rules_without_citizenship</t>
+    <t xml:space="preserve">Automated + Evaluation (30 real ads, author's labels)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest 21 Oct (137 passed): test_ad_requirements.py::test_live_job_requirements_read_by_the_rules_without_citizenship; E6 on 30 live ads not used to write the rules, labelled by the author (docs/evidence/ad_requirements/scores.txt, labels_author.csv)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As expected. Rules vs the author's labels on 30 real ads: qualification 28/30 (93%), field 29/30 (97%), languages 29/30 (97%), citizenship 28/30 (93%), salary 30/30 (100%); all above the bars set beforehand (90%; field 80%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E6 run 19 Oct; three AI judges as a cross-check only</t>
   </si>
   <si>
     <t xml:space="preserve">TC-19</t>
@@ -415,7 +424,16 @@
     <t xml:space="preserve">Employer posts shown as written; invented answers dropped</t>
   </si>
   <si>
-    <t xml:space="preserve">pytest 21 Oct (137 passed): test_description_grounding.py (3 tests)</t>
+    <t xml:space="preserve">Automated + Evaluation (real ads)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest 21 Oct (137 passed): test_description_grounding.py (3 tests); real-ad check 18 Oct: every saved description checked against its advert (docs/evidence/description_grounding.txt) and the 78 flagged bullets read against the full ad (description_grounding_flagged_labelled.csv)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As expected. 48 saved descriptions checked, 27 flagged; of the 78 flagged bullets: 27 invented (22 from an employer test post 'test ttt...'), 43 reworded but true, 8 translated from Malay and true. Invented bullets are now blocked and rebuilt; an employer's post is shown as written</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The 78 flagged bullets were labelled by Claude, not the author; a human check is planned (end of testing)</t>
   </si>
   <si>
     <t xml:space="preserve">TC-21</t>
@@ -1334,6 +1352,102 @@
   </si>
   <si>
     <t xml:space="preserve">The date is the promise to people who already applied; only 'Move decision date' changes it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code quality: linter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ruff check app tests tests_unit scripts migrations (Ruff's default rules: PEP 8 statements, unused imports, undefined names)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No findings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Ruff 0.15.11 (backend/ruff.toml)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/quality/ruff_26oct.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All checks passed! (first run: 62 findings, all style; fixed by hand or with reviewed fixes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One 'unsafe' automatic fix would have broken a database filter (SQLAlchemy != None); replaced by .is_not(None). See references.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security scan of SkillMap's own code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bandit -r app</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No High or Medium issues; every finding fixed or reviewed with the reason recorded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Bandit 1.9.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/quality/bandit_26oct.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No issues identified; 11 reviewed and skipped (# nosec with the test ID and reason). First run: 0 High, 2 Medium, 9 Low. Both Medium fixed: the model now loads from its own folder only (local_files_only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Libraries' known holes are TC-65 (pip-audit / npm audit); this row is our own code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-77</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python -m pytest -q --cov --cov-report=term (statements in app/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Above 60% ('acceptable'); aim 75% ('commendable'): Google Testing Blog, 2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: pytest-cov (backend/.coveragerc)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/quality/coverage_26oct.txt (184 passed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">75% of 6,402 statements. Lowest by design: embedder 0% (real SBERT replaced in tests), mailer, GitHub (no network); real gaps: admin_academic 45%, profile 64%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coverage shows what is not tested, not test quality (Google Testing Blog)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-78</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skill relation model beats plain cosine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SkillMap's trained relation model (DeBERTa-v3, 3 seeds averaged) vs cosine &gt;= 0.7 on a blind reference set of real module-skill / job-skill pairs judged by 3 people</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beats cosine and the previous model (rule set before the run)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/relation_model/reference_eval_esco_onet_v1_skillmap_v2_soft_skillmap_v3_soft_nli-deberta-v3-base_rw3x20_noextend_set4.json (run 6, commit 499d226)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanimous pairs (91): macro-F1 0.815 vs cosine 0.593; wrong 'has it' 9 vs 22. Majority pairs (132): 0.667 vs 0.516. Verdict: PASS, use the new model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The model in the app (RELATION_MODEL_DIR); evaluated before it went in</t>
   </si>
   <si>
     <t xml:space="preserve">SkillMap system testing — summary</t>
@@ -1851,7 +1965,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -2538,13 +2652,13 @@
         <v>118</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>27</v>
+        <v>119</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>29</v>
+        <v>121</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>21</v>
@@ -2552,11 +2666,13 @@
       <c r="K19" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="L19" s="3"/>
+      <c r="L19" s="3" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>103</v>
@@ -2565,19 +2681,19 @@
         <v>104</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>29</v>
@@ -2592,7 +2708,7 @@
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>103</v>
@@ -2601,22 +2717,22 @@
         <v>104</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>27</v>
+        <v>132</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>29</v>
+        <v>134</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>21</v>
@@ -2624,11 +2740,13 @@
       <c r="K21" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="L21" s="3"/>
+      <c r="L21" s="3" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>103</v>
@@ -2637,19 +2755,19 @@
         <v>104</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>29</v>
@@ -2664,28 +2782,28 @@
     </row>
     <row r="23" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>29</v>
@@ -2700,28 +2818,28 @@
     </row>
     <row r="24" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>136</v>
-      </c>
       <c r="C24" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>29</v>
@@ -2736,28 +2854,28 @@
     </row>
     <row r="25" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>29</v>
@@ -2772,28 +2890,28 @@
     </row>
     <row r="26" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>29</v>
@@ -2808,64 +2926,64 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="L27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="I28" s="3" t="s">
         <v>29</v>
@@ -2880,28 +2998,28 @@
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>76</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>29</v>
@@ -2916,28 +3034,28 @@
     </row>
     <row r="30" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>177</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>171</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>76</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>29</v>
@@ -2952,28 +3070,28 @@
     </row>
     <row r="31" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>76</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>29</v>
@@ -2988,28 +3106,28 @@
     </row>
     <row r="32" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>76</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>29</v>
@@ -3024,28 +3142,28 @@
     </row>
     <row r="33" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>76</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="I33" s="3" t="s">
         <v>29</v>
@@ -3060,28 +3178,28 @@
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>76</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="I34" s="3" t="s">
         <v>29</v>
@@ -3096,28 +3214,28 @@
     </row>
     <row r="35" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>76</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>29</v>
@@ -3132,28 +3250,28 @@
     </row>
     <row r="36" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>29</v>
@@ -3168,28 +3286,28 @@
     </row>
     <row r="37" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>208</v>
-      </c>
       <c r="C37" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="I37" s="3" t="s">
         <v>29</v>
@@ -3204,28 +3322,28 @@
     </row>
     <row r="38" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="I38" s="3" t="s">
         <v>29</v>
@@ -3234,36 +3352,36 @@
         <v>21</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>29</v>
@@ -3278,28 +3396,28 @@
     </row>
     <row r="40" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="I40" s="3" t="s">
         <v>29</v>
@@ -3314,28 +3432,28 @@
     </row>
     <row r="41" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="G41" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="I41" s="3" t="s">
         <v>29</v>
@@ -3350,28 +3468,28 @@
     </row>
     <row r="42" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="I42" s="3" t="s">
         <v>29</v>
@@ -3386,28 +3504,28 @@
     </row>
     <row r="43" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>29</v>
@@ -3422,28 +3540,28 @@
     </row>
     <row r="44" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="I44" s="3" t="s">
         <v>29</v>
@@ -3452,34 +3570,34 @@
         <v>21</v>
       </c>
       <c r="K44" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="L44" s="3"/>
     </row>
     <row r="45" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>29</v>
@@ -3494,28 +3612,28 @@
     </row>
     <row r="46" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="I46" s="3" t="s">
         <v>29</v>
@@ -3530,28 +3648,28 @@
     </row>
     <row r="47" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>29</v>
@@ -3566,28 +3684,28 @@
     </row>
     <row r="48" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="I48" s="3" t="s">
         <v>29</v>
@@ -3602,28 +3720,28 @@
     </row>
     <row r="49" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="I49" s="3" t="s">
         <v>29</v>
@@ -3638,28 +3756,28 @@
     </row>
     <row r="50" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="I50" s="3" t="s">
         <v>29</v>
@@ -3674,31 +3792,31 @@
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>18</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="J51" s="3" t="s">
         <v>21</v>
@@ -3710,28 +3828,28 @@
     </row>
     <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="I52" s="3" t="s">
         <v>29</v>
@@ -3746,28 +3864,28 @@
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="I53" s="3" t="s">
         <v>29</v>
@@ -3782,64 +3900,64 @@
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="J54" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K54" s="3" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="L54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="I55" s="3" t="s">
         <v>29</v>
@@ -3851,33 +3969,33 @@
         <v>22</v>
       </c>
       <c r="L55" s="3" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="B56" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="B56" s="3" t="s">
-        <v>311</v>
-      </c>
       <c r="C56" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="I56" s="3" t="s">
         <v>29</v>
@@ -3892,28 +4010,28 @@
     </row>
     <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="I57" s="3" t="s">
         <v>29</v>
@@ -3928,28 +4046,28 @@
     </row>
     <row r="58" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="I58" s="3" t="s">
         <v>29</v>
@@ -3964,28 +4082,28 @@
     </row>
     <row r="59" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="I59" s="3" t="s">
         <v>29</v>
@@ -4000,28 +4118,28 @@
     </row>
     <row r="60" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="I60" s="3" t="s">
         <v>29</v>
@@ -4036,28 +4154,28 @@
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="I61" s="3" t="s">
         <v>29</v>
@@ -4072,28 +4190,28 @@
     </row>
     <row r="62" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="I62" s="3" t="s">
         <v>29</v>
@@ -4108,28 +4226,28 @@
     </row>
     <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="I63" s="3" t="s">
         <v>29</v>
@@ -4144,28 +4262,28 @@
     </row>
     <row r="64" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="I64" s="3" t="s">
         <v>29</v>
@@ -4180,67 +4298,67 @@
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="J65" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K65" s="3" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="L65" s="3"/>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="J66" s="3" t="s">
         <v>21</v>
@@ -4252,170 +4370,170 @@
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="J67" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K67" s="3" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="L67" s="3"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="H68" s="3"/>
       <c r="I68" s="3"/>
       <c r="J68" s="3" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="K68" s="3"/>
       <c r="L68" s="3"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="J69" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K69" s="3" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="L69" s="3" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="J70" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K70" s="3" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="L70" s="3" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="G71" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="I71" s="3" t="s">
         <v>29</v>
@@ -4424,36 +4542,36 @@
         <v>21</v>
       </c>
       <c r="K71" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="L71" s="3" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="G72" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="I72" s="3" t="s">
         <v>29</v>
@@ -4462,34 +4580,34 @@
         <v>21</v>
       </c>
       <c r="K72" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="L72" s="3"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="G73" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="I73" s="3" t="s">
         <v>29</v>
@@ -4498,36 +4616,36 @@
         <v>21</v>
       </c>
       <c r="K73" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="L73" s="3" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="G74" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="I74" s="3" t="s">
         <v>29</v>
@@ -4536,36 +4654,36 @@
         <v>21</v>
       </c>
       <c r="K74" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="L74" s="3" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="G75" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="I75" s="3" t="s">
         <v>29</v>
@@ -4574,14 +4692,166 @@
         <v>21</v>
       </c>
       <c r="K75" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="L75" s="3" t="s">
-        <v>435</v>
+        <v>441</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="J76" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K76" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="L76" s="3" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="E77" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="G77" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="I77" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="J77" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K77" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="L77" s="3" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="I78" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="J78" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K78" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="L78" s="3" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="I79" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K79" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="L79" s="3" t="s">
+        <v>473</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L75"/>
+  <autoFilter ref="A1:L79"/>
   <conditionalFormatting sqref="J2:J100">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Fail"</formula>
@@ -4621,12 +4891,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>436</v>
+        <v>474</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>437</v>
+        <v>475</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4634,16 +4904,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>438</v>
+        <v>476</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>439</v>
+        <v>477</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4694,11 +4964,11 @@
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A7)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$100,$A7,'Test cases'!$J$2:$J$100,"Pass")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$100,$A7,'Test cases'!$J$2:$J$100,"Fail")</f>
@@ -4732,7 +5002,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A9)</f>
@@ -4753,7 +5023,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A10)</f>
@@ -4774,7 +5044,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A11)</f>
@@ -4795,7 +5065,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A12)</f>
@@ -4816,7 +5086,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="B13" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A13)</f>
@@ -4837,7 +5107,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="B14" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A14)</f>
@@ -4858,7 +5128,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="B15" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A15)</f>
@@ -4879,15 +5149,15 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="B16" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A16)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$100,$A16,'Test cases'!$J$2:$J$100,"Pass")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$100,$A16,'Test cases'!$J$2:$J$100,"Fail")</f>
@@ -4900,15 +5170,15 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>438</v>
+        <v>476</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">SUM(B5:B16)</f>
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">SUM(C5:C16)</f>
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D17" s="8" t="n">
         <f aca="false">SUM(D5:D16)</f>
@@ -4928,7 +5198,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>440</v>
+        <v>478</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -4937,7 +5207,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>441</v>
+        <v>479</v>
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"1")</f>
@@ -4952,22 +5222,22 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>442</v>
+        <v>480</v>
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"2")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C21" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$C$2:$C$100,"2",'Test cases'!$J$2:$J$100,"Pass")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D21" s="7"/>
       <c r="E21" s="7"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>443</v>
+        <v>481</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"3")</f>
@@ -4982,7 +5252,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>444</v>
+        <v>482</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"4")</f>
@@ -5026,42 +5296,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>445</v>
+        <v>483</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>446</v>
+        <v>484</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>447</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>448</v>
+        <v>486</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>449</v>
+        <v>487</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>450</v>
+        <v>488</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>451</v>
+        <v>489</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>452</v>
+        <v>490</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Docker: compose (db, mongo, api, web), Dockerfiles, restore script, smoke test; workbook TC-79 to TC-81; README, CHANGELOG, roadmap and references brought up to date for 23-28 Oct
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Test cases'!$1:$1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Test cases'!$A$1:$L$79</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Test cases'!$A$1:$L$82</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="518">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1207,18 +1207,24 @@
     <t xml:space="preserve">Runs the same in Docker</t>
   </si>
   <si>
-    <t xml:space="preserve">Build the Docker images, run the tests inside</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same results as on the laptop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool (step 5)</t>
+    <t xml:space="preserve">docker compose up --build (first start restores docker/db/skillmap.dump), wait until the backend is healthy, then from backend/: python scripts/tools/docker_smoke.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All 9 checks pass: API answers, CORS for the web app, web app and a deep link served, built JavaScript served, job data present, student can register and sign in, a signed-in call reads the database, the account can be deleted, an idle connection stays open for 7 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Docker Compose + backend/scripts/tools/docker_smoke.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/docker/ (smoke output to be saved after the run)</t>
   </si>
   <si>
     <t xml:space="preserve">Not run</t>
   </si>
   <si>
+    <t xml:space="preserve">Built 28 Oct. The smoke script was tested against a stand-in server (9 of 9; check 9 fails on a 2 s keep-alive). The images have not been built or run yet</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC-68</t>
   </si>
   <si>
@@ -1448,6 +1454,81 @@
   </si>
   <si>
     <t xml:space="preserve">The model in the app (RELATION_MODEL_DIR); evaluated before it went in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load: 5, 10 and 20 students at the same time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python scripts/evaluation/evaluate_load.py (one uvicorn process; Locust students open Job Matches, Job Detail and the Dashboard with a 3-10 s pause; 3 minutes per stage)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No failed call and every call's p95 under 1 s (rule fixed before the first run; 1 s = Nielsen's limit for keeping the flow of thought)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Locust 2.47.0 (backend/scripts/evaluation/evaluate_load.py)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/performance/load/summary.txt (run 3); runs 1 and 2 in docs/evidence/performance/load_runs/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run 3: 0 failed calls at 5 students (488 calls), 10 (884) and 20 (1,781 calls, 9.9 calls/s). Slowest call POST /recommend/: p95 0.49 / 0.52 / 0.92 s. Runs 1 and 2 passed these stages too</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comfortable capacity = 20 students (about 10 calls/s); POST /recommend/ p95 at 20 students was 0.45-0.92 s over the three runs, so 20 is the limit, not a wide margin. One laptop runs the server, the database and the load generator; the pauses are assumed, not measured. Server CPU in run 1 was measured on the launcher process (0%), fixed from run 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load: 40 students, no failed call</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same script, 40-student stage (3 minutes), then a stress stage of 20 students with almost no pause (0.2-0.5 s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No failed call and every call's p95 under 10 s (Nielsen's attention limit); the stress stage has no rule and shows where the server gives in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/performance/load/summary.txt (run 3); docs/evidence/performance/load_runs/run1 and run2 (the two failing runs, with server.log)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run 1 (uvicorn default keep-alive): FAIL, 1 of 3,598 calls failed. Run 2 (default): FAIL, 4 of 3,606 failed. All 5 were GET /auth/me, RemoteDisconnected; the server log showed no error. Run 3 (--timeout-keep-alive 15): 0 of 3,411 failed, slowest p95 POST /recommend/ 2.8 s. Stress: 0 failures, 27.7 calls/s, POST /recommend/ p95 3.7 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only the server setting changed between runs 2 and 3, not the rule. Likely cause: uvicorn closes idle connections after 5 s (its documented default) and the simulated pauses run to 10 s; a stand-in server with a 2 s keep-alive and a 4 s idle gap reproduced RemoteDisconnected (docker_smoke.py check 9). The start command and Docker use 15 s. Cause not proven on the real server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Front-end unit tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From frontend/: npm test (Vitest 5.0.5, jsdom, Testing Library); npm run test:coverage for the table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All tests pass; each rule is checked by breaking it on purpose and seeing a test fail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Vitest + Testing Library</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/tests/vitest_2026-10-28.txt, vitest_coverage_2026-10-28.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 files, 101 tests passed on Windows. Covers: sign-in expiry and 422 handling (api.js), the saved-answer cache (15 minutes, dropped on a profile change), live password guidance (length only, common list, 72 bytes), level tag, confirm box, info tip, toast, skill names, greeting, profile checklist, admin decisions, employer statuses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coverage of the whole front-end is 3.7%: pages are covered by the 18 browser tests and the axe and Lighthouse scans; Vitest covers logic and small components (94-100% of lines in the files it tests). Ten rules were broken on purpose and all were caught</t>
   </si>
   <si>
     <t xml:space="preserve">SkillMap system testing — summary</t>
@@ -1965,7 +2046,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -4426,17 +4507,21 @@
       <c r="G68" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="H68" s="3"/>
+      <c r="H68" s="3" t="s">
+        <v>396</v>
+      </c>
       <c r="I68" s="3"/>
       <c r="J68" s="3" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="K68" s="3"/>
-      <c r="L68" s="3"/>
+      <c r="L68" s="3" t="s">
+        <v>398</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>376</v>
@@ -4445,22 +4530,22 @@
         <v>215</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="J69" s="3" t="s">
         <v>21</v>
@@ -4469,12 +4554,12 @@
         <v>390</v>
       </c>
       <c r="L69" s="3" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>349</v>
@@ -4483,22 +4568,22 @@
         <v>143</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="J70" s="3" t="s">
         <v>21</v>
@@ -4507,12 +4592,12 @@
         <v>390</v>
       </c>
       <c r="L70" s="3" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>214</v>
@@ -4521,19 +4606,19 @@
         <v>215</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="G71" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="I71" s="3" t="s">
         <v>29</v>
@@ -4545,12 +4630,12 @@
         <v>230</v>
       </c>
       <c r="L71" s="3" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>214</v>
@@ -4559,19 +4644,19 @@
         <v>215</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G72" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="I72" s="3" t="s">
         <v>29</v>
@@ -4586,7 +4671,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>214</v>
@@ -4595,19 +4680,19 @@
         <v>215</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="G73" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="I73" s="3" t="s">
         <v>29</v>
@@ -4619,12 +4704,12 @@
         <v>230</v>
       </c>
       <c r="L73" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>214</v>
@@ -4633,19 +4718,19 @@
         <v>215</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="G74" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="I74" s="3" t="s">
         <v>29</v>
@@ -4657,12 +4742,12 @@
         <v>230</v>
       </c>
       <c r="L74" s="3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>214</v>
@@ -4671,19 +4756,19 @@
         <v>215</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="G75" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="I75" s="3" t="s">
         <v>29</v>
@@ -4695,12 +4780,12 @@
         <v>230</v>
       </c>
       <c r="L75" s="3" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>376</v>
@@ -4709,22 +4794,22 @@
         <v>215</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="J76" s="3" t="s">
         <v>21</v>
@@ -4733,12 +4818,12 @@
         <v>230</v>
       </c>
       <c r="L76" s="3" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>376</v>
@@ -4747,22 +4832,22 @@
         <v>215</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="I77" s="3" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="J77" s="3" t="s">
         <v>21</v>
@@ -4771,12 +4856,12 @@
         <v>230</v>
       </c>
       <c r="L77" s="3" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>376</v>
@@ -4785,22 +4870,22 @@
         <v>215</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="H78" s="3" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="J78" s="3" t="s">
         <v>21</v>
@@ -4809,12 +4894,12 @@
         <v>230</v>
       </c>
       <c r="L78" s="3" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>75</v>
@@ -4823,35 +4908,149 @@
         <v>76</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="G79" s="3" t="s">
         <v>45</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="J79" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K79" s="3" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="L79" s="3" t="s">
-        <v>473</v>
+        <v>475</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="E80" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="F80" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="G80" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="H80" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="I80" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="J80" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K80" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="L80" s="3" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="F81" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="G81" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="H81" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="I81" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="J81" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K81" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="L81" s="3" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="E82" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="F82" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="G82" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="I82" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="J82" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K82" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="L82" s="3" t="s">
+        <v>500</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L79"/>
+  <autoFilter ref="A1:L82"/>
   <conditionalFormatting sqref="J2:J100">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Fail"</formula>
@@ -4891,12 +5090,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>474</v>
+        <v>501</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>475</v>
+        <v>502</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4904,16 +5103,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>476</v>
+        <v>503</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>477</v>
+        <v>504</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5153,11 +5352,11 @@
       </c>
       <c r="B16" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$B$2:$B$100,A16)</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$100,$A16,'Test cases'!$J$2:$J$100,"Pass")</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$100,$A16,'Test cases'!$J$2:$J$100,"Fail")</f>
@@ -5170,15 +5369,15 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>476</v>
+        <v>503</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">SUM(B5:B16)</f>
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">SUM(C5:C16)</f>
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D17" s="8" t="n">
         <f aca="false">SUM(D5:D16)</f>
@@ -5198,7 +5397,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>478</v>
+        <v>505</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -5207,7 +5406,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>479</v>
+        <v>506</v>
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"1")</f>
@@ -5222,7 +5421,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>480</v>
+        <v>507</v>
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"2")</f>
@@ -5237,7 +5436,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>481</v>
+        <v>508</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"3")</f>
@@ -5252,7 +5451,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>482</v>
+        <v>509</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"4")</f>
@@ -5296,42 +5495,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>483</v>
+        <v>510</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>484</v>
+        <v>511</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>485</v>
+        <v>512</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>486</v>
+        <v>513</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>487</v>
+        <v>514</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>488</v>
+        <v>515</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>489</v>
+        <v>516</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>490</v>
+        <v>517</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Docker: first Windows run passes (TC-67, 9 of 9 smoke checks); workbook 81/81; smoke script reports connection errors as FAIL; md files updated
</commit_message>
<xml_diff>
--- a/docs/testing/SkillMap_system_test_cases.xlsx
+++ b/docs/testing/SkillMap_system_test_cases.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="520">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1216,331 +1216,337 @@
     <t xml:space="preserve">Tool: Docker Compose + backend/scripts/tools/docker_smoke.py</t>
   </si>
   <si>
-    <t xml:space="preserve">docs/evidence/docker/ (smoke output to be saved after the run)</t>
+    <t xml:space="preserve">docs/evidence/docker/smoke_2026-10-29.txt, compose_ps_2026-10-29.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Docker Desktop on Windows, docker compose up --build: db (postgres:18), mongo (mongo:9) and backend healthy, frontend up. docker_smoke.py: 9 of 9 checks passed (API answers, CORS for the web app, web app and /login deep link, built JavaScript, 14 job categories, register and sign in, database read, delete account, idle connection open for 7 s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built 28 Oct, first run 29 Oct. The database image had to be PostgreSQL 18 (and the data volume mounted at /var/lib/postgresql) to restore a dump made on the laptop's PostgreSQL 18; MongoDB 9 to match. Check 9 passes because the start command sets --timeout-keep-alive 15. Chats made outside Docker are not in the container's MongoDB (only the PostgreSQL dump is restored). Containers run as root: laptop and demo use only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Works in other browsers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run the 18 browser tests in Chromium, Google Chrome, Microsoft Edge, Firefox and WebKit (Safari's engine): frontend/scripts/all_browsers.sh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All tests pass in each browser; applying confirmed within 1 s (Google RAIL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Playwright E2E (5 browsers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/e2e/run_2026-10-23.txt and firefox/, webkit/, edge/, chrome/ (run logs, results, screenshots, accessibility scans)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 of 18 in every browser (23 Oct, after the stale-answer fixes). Click to "Applied": Chromium 239 ms, Firefox 485 ms, WebKit 581 ms, Edge 239 ms, Chrome 454 ms (limit 1 s). In WebKit the keyboard tests focus the link directly (WebKit, like Safari, leaves links out of Tab by default)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not tested on real Safari (no Mac); WebKit is its engine. Phones and tablets out of scope (designed for laptops)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MongoDB for real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With MongoDB running: python -m pytest tests/test_mongodb_real.py (a separate skillmap_test database)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indexes incl. the 18-month expiry exist; a chat is saved, listed, reopened, continued and deleted; another student can't reach it; Download my data and Delete my account cover MongoDB; an evaluation run is saved and read back</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automated (real MongoDB server)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest 23 Oct (176 passed): docs/evidence/tests/pytest_2026-10-23.txt, tests/test_mongodb_real.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As expected: 4 of 4 against the real server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skipped with a message when MongoDB is off; the other tests use stand-ins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Declining an invitation, with or without a reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Student says No thanks with 'Already have an offer'; another with no reason; another picks 'Other' with no words; then one applies anyway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employer sees 'Declined · Already have an offer' and 'Declined · No reason given'; 'Other' without words refused; she can still apply, and that application is not tagged 'Invited'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_invitations.py::test_declining_shows_the_reason_and_still_lets_her_apply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reason optional; 'Other' needs words (up to 200 characters)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No answer in 14 days shows 'No reply'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invitation left unanswered for 15 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employer sees 'No reply'; the student no longer sees the invitation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_invitations.py::test_no_answer_after_14_days_is_no_reply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invite several at once</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tick graduates on View applicants (one already invited, one who has applied) and press Invite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each ticked graduate who can be invited is invited; the others are skipped and counted; at most 50 at a time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_invitations.py::test_invite_selected_invites_each_and_reports_the_rest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only graduates the employer ticks; no 'invite all' across jobs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-73</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Graduates who fit: order and nice-to-have skills</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two graduates with the same required skills, one also with the nice-to-have; then invite the better match</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The one with the nice-to-have comes first; employers see only the nice-to-haves a graduate has, never how many they lack; once invited, the graduate moves below those not invited yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_invitations.py::test_graduates_with_nice_to_have_skills_come_first, test_graduates_not_yet_invited_come_first</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Her 21 Oct rule: strengths only, never a 'no' that isn't required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taking applications again only before the decision date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stop new applications, take them again, stop again; then the decision date passes and try again</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stopping and restarting never move the decision date; restarting after the date has passed is refused</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_transparency.py::test_applications_can_restart_only_before_the_decision_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The date is the promise to people who already applied; only 'Move decision date' changes it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code quality: linter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ruff check app tests tests_unit scripts migrations (Ruff's default rules: PEP 8 statements, unused imports, undefined names)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No findings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Ruff 0.15.11 (backend/ruff.toml)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/quality/ruff_26oct.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All checks passed! (first run: 62 findings, all style; fixed by hand or with reviewed fixes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One 'unsafe' automatic fix would have broken a database filter (SQLAlchemy != None); replaced by .is_not(None). See references.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security scan of SkillMap's own code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bandit -r app</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No High or Medium issues; every finding fixed or reviewed with the reason recorded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Bandit 1.9.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/quality/bandit_26oct.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No issues identified; 11 reviewed and skipped (# nosec with the test ID and reason). First run: 0 High, 2 Medium, 9 Low. Both Medium fixed: the model now loads from its own folder only (local_files_only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Libraries' known holes are TC-65 (pip-audit / npm audit); this row is our own code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-77</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python -m pytest -q --cov --cov-report=term (statements in app/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Above 60% ('acceptable'); aim 75% ('commendable'): Google Testing Blog, 2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: pytest-cov (backend/.coveragerc)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/quality/coverage_26oct.txt (184 passed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">75% of 6,402 statements. Lowest by design: embedder 0% (real SBERT replaced in tests), mailer, GitHub (no network); real gaps: admin_academic 45%, profile 64%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coverage shows what is not tested, not test quality (Google Testing Blog)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-78</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skill relation model beats plain cosine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SkillMap's trained relation model (DeBERTa-v3, 3 seeds averaged) vs cosine &gt;= 0.7 on a blind reference set of real module-skill / job-skill pairs judged by 3 people</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beats cosine and the previous model (rule set before the run)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/relation_model/reference_eval_esco_onet_v1_skillmap_v2_soft_skillmap_v3_soft_nli-deberta-v3-base_rw3x20_noextend_set4.json (run 6, commit 499d226)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanimous pairs (91): macro-F1 0.815 vs cosine 0.593; wrong 'has it' 9 vs 22. Majority pairs (132): 0.667 vs 0.516. Verdict: PASS, use the new model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The model in the app (RELATION_MODEL_DIR); evaluated before it went in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load: 5, 10 and 20 students at the same time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python scripts/evaluation/evaluate_load.py (one uvicorn process; Locust students open Job Matches, Job Detail and the Dashboard with a 3-10 s pause; 3 minutes per stage)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No failed call and every call's p95 under 1 s (rule fixed before the first run; 1 s = Nielsen's limit for keeping the flow of thought)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Locust 2.47.0 (backend/scripts/evaluation/evaluate_load.py)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/performance/load/summary.txt (run 3); runs 1 and 2 in docs/evidence/performance/load_runs/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run 3: 0 failed calls at 5 students (488 calls), 10 (884) and 20 (1,781 calls, 9.9 calls/s). Slowest call POST /recommend/: p95 0.49 / 0.52 / 0.92 s. Runs 1 and 2 passed these stages too</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comfortable capacity = 20 students (about 10 calls/s); POST /recommend/ p95 at 20 students was 0.45-0.92 s over the three runs, so 20 is the limit, not a wide margin. One laptop runs the server, the database and the load generator; the pauses are assumed, not measured. Server CPU in run 1 was measured on the launcher process (0%), fixed from run 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load: 40 students, no failed call</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same script, 40-student stage (3 minutes), then a stress stage of 20 students with almost no pause (0.2-0.5 s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No failed call and every call's p95 under 10 s (Nielsen's attention limit); the stress stage has no rule and shows where the server gives in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/performance/load/summary.txt (run 3); docs/evidence/performance/load_runs/run1 and run2 (the two failing runs, with server.log)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run 1 (uvicorn default keep-alive): FAIL, 1 of 3,598 calls failed. Run 2 (default): FAIL, 4 of 3,606 failed. All 5 were GET /auth/me, RemoteDisconnected; the server log showed no error. Run 3 (--timeout-keep-alive 15): 0 of 3,411 failed, slowest p95 POST /recommend/ 2.8 s. Stress: 0 failures, 27.7 calls/s, POST /recommend/ p95 3.7 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only the server setting changed between runs 2 and 3, not the rule. Likely cause: uvicorn closes idle connections after 5 s (its documented default) and the simulated pauses run to 10 s; a stand-in server with a 2 s keep-alive and a 4 s idle gap reproduced RemoteDisconnected (docker_smoke.py check 9). The start command and Docker use 15 s. Cause not proven on the real server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Front-end unit tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From frontend/: npm test (Vitest 5.0.5, jsdom, Testing Library); npm run test:coverage for the table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All tests pass; each rule is checked by breaking it on purpose and seeing a test fail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool: Vitest + Testing Library</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/tests/vitest_2026-10-28.txt, vitest_coverage_2026-10-28.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 files, 101 tests passed on Windows. Covers: sign-in expiry and 422 handling (api.js), the saved-answer cache (15 minutes, dropped on a profile change), live password guidance (length only, common list, 72 bytes), level tag, confirm box, info tip, toast, skill names, greeting, profile checklist, admin decisions, employer statuses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coverage of the whole front-end is 3.7%: pages are covered by the 18 browser tests and the axe and Lighthouse scans; Vitest covers logic and small components (94-100% of lines in the files it tests). Ten rules were broken on purpose and all were caught</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SkillMap system testing — summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counts update from the Status column of 'Test cases'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fail</t>
   </si>
   <si>
     <t xml:space="preserve">Not run</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Built 28 Oct. The smoke script was tested against a stand-in server (9 of 9; check 9 fails on a 2 s keep-alive). The images have not been built or run yet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-68</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Works in other browsers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run the 18 browser tests in Chromium, Google Chrome, Microsoft Edge, Firefox and WebKit (Safari's engine): frontend/scripts/all_browsers.sh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All tests pass in each browser; applying confirmed within 1 s (Google RAIL)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Playwright E2E (5 browsers)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/evidence/e2e/run_2026-10-23.txt and firefox/, webkit/, edge/, chrome/ (run logs, results, screenshots, accessibility scans)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18 of 18 in every browser (23 Oct, after the stale-answer fixes). Click to "Applied": Chromium 239 ms, Firefox 485 ms, WebKit 581 ms, Edge 239 ms, Chrome 454 ms (limit 1 s). In WebKit the keyboard tests focus the link directly (WebKit, like Safari, leaves links out of Tab by default)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not tested on real Safari (no Mac); WebKit is its engine. Phones and tablets out of scope (designed for laptops)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-69</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MongoDB for real</t>
-  </si>
-  <si>
-    <t xml:space="preserve">With MongoDB running: python -m pytest tests/test_mongodb_real.py (a separate skillmap_test database)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indexes incl. the 18-month expiry exist; a chat is saved, listed, reopened, continued and deleted; another student can't reach it; Download my data and Delete my account cover MongoDB; an evaluation run is saved and read back</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automated (real MongoDB server)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pytest 23 Oct (176 passed): docs/evidence/tests/pytest_2026-10-23.txt, tests/test_mongodb_real.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As expected: 4 of 4 against the real server</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skipped with a message when MongoDB is off; the other tests use stand-ins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-70</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Declining an invitation, with or without a reason</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Student says No thanks with 'Already have an offer'; another with no reason; another picks 'Other' with no words; then one applies anyway</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employer sees 'Declined · Already have an offer' and 'Declined · No reason given'; 'Other' without words refused; she can still apply, and that application is not tagged 'Invited'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_invitations.py::test_declining_shows_the_reason_and_still_lets_her_apply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reason optional; 'Other' needs words (up to 200 characters)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-71</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No answer in 14 days shows 'No reply'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invitation left unanswered for 15 days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employer sees 'No reply'; the student no longer sees the invitation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_invitations.py::test_no_answer_after_14_days_is_no_reply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-72</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invite several at once</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tick graduates on View applicants (one already invited, one who has applied) and press Invite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each ticked graduate who can be invited is invited; the others are skipped and counted; at most 50 at a time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_invitations.py::test_invite_selected_invites_each_and_reports_the_rest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only graduates the employer ticks; no 'invite all' across jobs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-73</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Graduates who fit: order and nice-to-have skills</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Two graduates with the same required skills, one also with the nice-to-have; then invite the better match</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The one with the nice-to-have comes first; employers see only the nice-to-haves a graduate has, never how many they lack; once invited, the graduate moves below those not invited yet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_invitations.py::test_graduates_with_nice_to_have_skills_come_first, test_graduates_not_yet_invited_come_first</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Her 21 Oct rule: strengths only, never a 'no' that isn't required</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-74</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taking applications again only before the decision date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stop new applications, take them again, stop again; then the decision date passes and try again</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stopping and restarting never move the decision date; restarting after the date has passed is refused</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pytest 26 Oct (184 passed): docs/evidence/tests/pytest_26oct.txt: test_transparency.py::test_applications_can_restart_only_before_the_decision_date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The date is the promise to people who already applied; only 'Move decision date' changes it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code quality: linter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ruff check app tests tests_unit scripts migrations (Ruff's default rules: PEP 8 statements, unused imports, undefined names)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No findings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool: Ruff 0.15.11 (backend/ruff.toml)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/evidence/quality/ruff_26oct.txt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All checks passed! (first run: 62 findings, all style; fixed by hand or with reviewed fixes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One 'unsafe' automatic fix would have broken a database filter (SQLAlchemy != None); replaced by .is_not(None). See references.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-76</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Security scan of SkillMap's own code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bandit -r app</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No High or Medium issues; every finding fixed or reviewed with the reason recorded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool: Bandit 1.9.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/evidence/quality/bandit_26oct.txt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No issues identified; 11 reviewed and skipped (# nosec with the test ID and reason). First run: 0 High, 2 Medium, 9 Low. Both Medium fixed: the model now loads from its own folder only (local_files_only)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Libraries' known holes are TC-65 (pip-audit / npm audit); this row is our own code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-77</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test coverage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">python -m pytest -q --cov --cov-report=term (statements in app/)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Above 60% ('acceptable'); aim 75% ('commendable'): Google Testing Blog, 2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool: pytest-cov (backend/.coveragerc)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/evidence/quality/coverage_26oct.txt (184 passed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">75% of 6,402 statements. Lowest by design: embedder 0% (real SBERT replaced in tests), mailer, GitHub (no network); real gaps: admin_academic 45%, profile 64%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coverage shows what is not tested, not test quality (Google Testing Blog)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-78</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skill relation model beats plain cosine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SkillMap's trained relation model (DeBERTa-v3, 3 seeds averaged) vs cosine &gt;= 0.7 on a blind reference set of real module-skill / job-skill pairs judged by 3 people</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beats cosine and the previous model (rule set before the run)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/evidence/relation_model/reference_eval_esco_onet_v1_skillmap_v2_soft_skillmap_v3_soft_nli-deberta-v3-base_rw3x20_noextend_set4.json (run 6, commit 499d226)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unanimous pairs (91): macro-F1 0.815 vs cosine 0.593; wrong 'has it' 9 vs 22. Majority pairs (132): 0.667 vs 0.516. Verdict: PASS, use the new model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 Oct 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The model in the app (RELATION_MODEL_DIR); evaluated before it went in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-79</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Load: 5, 10 and 20 students at the same time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">python scripts/evaluation/evaluate_load.py (one uvicorn process; Locust students open Job Matches, Job Detail and the Dashboard with a 3-10 s pause; 3 minutes per stage)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No failed call and every call's p95 under 1 s (rule fixed before the first run; 1 s = Nielsen's limit for keeping the flow of thought)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool: Locust 2.47.0 (backend/scripts/evaluation/evaluate_load.py)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/evidence/performance/load/summary.txt (run 3); runs 1 and 2 in docs/evidence/performance/load_runs/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run 3: 0 failed calls at 5 students (488 calls), 10 (884) and 20 (1,781 calls, 9.9 calls/s). Slowest call POST /recommend/: p95 0.49 / 0.52 / 0.92 s. Runs 1 and 2 passed these stages too</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27 Oct 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comfortable capacity = 20 students (about 10 calls/s); POST /recommend/ p95 at 20 students was 0.45-0.92 s over the three runs, so 20 is the limit, not a wide margin. One laptop runs the server, the database and the load generator; the pauses are assumed, not measured. Server CPU in run 1 was measured on the launcher process (0%), fixed from run 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Load: 40 students, no failed call</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same script, 40-student stage (3 minutes), then a stress stage of 20 students with almost no pause (0.2-0.5 s)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No failed call and every call's p95 under 10 s (Nielsen's attention limit); the stress stage has no rule and shows where the server gives in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/evidence/performance/load/summary.txt (run 3); docs/evidence/performance/load_runs/run1 and run2 (the two failing runs, with server.log)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run 1 (uvicorn default keep-alive): FAIL, 1 of 3,598 calls failed. Run 2 (default): FAIL, 4 of 3,606 failed. All 5 were GET /auth/me, RemoteDisconnected; the server log showed no error. Run 3 (--timeout-keep-alive 15): 0 of 3,411 failed, slowest p95 POST /recommend/ 2.8 s. Stress: 0 failures, 27.7 calls/s, POST /recommend/ p95 3.7 s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only the server setting changed between runs 2 and 3, not the rule. Likely cause: uvicorn closes idle connections after 5 s (its documented default) and the simulated pauses run to 10 s; a stand-in server with a 2 s keep-alive and a 4 s idle gap reproduced RemoteDisconnected (docker_smoke.py check 9). The start command and Docker use 15 s. Cause not proven on the real server</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-81</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Front-end unit tests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">From frontend/: npm test (Vitest 5.0.5, jsdom, Testing Library); npm run test:coverage for the table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All tests pass; each rule is checked by breaking it on purpose and seeing a test fail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool: Vitest + Testing Library</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/evidence/tests/vitest_2026-10-28.txt, vitest_coverage_2026-10-28.txt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 files, 101 tests passed on Windows. Covers: sign-in expiry and 422 handling (api.js), the saved-answer cache (15 minutes, dropped on a profile change), live password guidance (length only, common list, 72 bytes), level tag, confirm box, info tip, toast, skill names, greeting, profile checklist, admin decisions, employer statuses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28 Oct 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coverage of the whole front-end is 3.7%: pages are covered by the 18 browser tests and the axe and Lighthouse scans; Vitest covers logic and small components (94-100% of lines in the files it tests). Ten rules were broken on purpose and all were caught</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SkillMap system testing — summary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Counts update from the Status column of 'Test cases'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fail</t>
   </si>
   <si>
     <t xml:space="preserve">By IR objective</t>
@@ -4510,18 +4516,22 @@
       <c r="H68" s="3" t="s">
         <v>396</v>
       </c>
-      <c r="I68" s="3"/>
+      <c r="I68" s="3" t="s">
+        <v>397</v>
+      </c>
       <c r="J68" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="K68" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="K68" s="3" t="s">
+        <v>398</v>
+      </c>
       <c r="L68" s="3" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>376</v>
@@ -4530,22 +4540,22 @@
         <v>215</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="J69" s="3" t="s">
         <v>21</v>
@@ -4554,12 +4564,12 @@
         <v>390</v>
       </c>
       <c r="L69" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>349</v>
@@ -4568,22 +4578,22 @@
         <v>143</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J70" s="3" t="s">
         <v>21</v>
@@ -4592,12 +4602,12 @@
         <v>390</v>
       </c>
       <c r="L70" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>214</v>
@@ -4606,19 +4616,19 @@
         <v>215</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G71" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="I71" s="3" t="s">
         <v>29</v>
@@ -4630,12 +4640,12 @@
         <v>230</v>
       </c>
       <c r="L71" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>214</v>
@@ -4644,19 +4654,19 @@
         <v>215</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G72" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="I72" s="3" t="s">
         <v>29</v>
@@ -4671,7 +4681,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>214</v>
@@ -4680,19 +4690,19 @@
         <v>215</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="G73" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I73" s="3" t="s">
         <v>29</v>
@@ -4704,12 +4714,12 @@
         <v>230</v>
       </c>
       <c r="L73" s="3" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>214</v>
@@ -4718,19 +4728,19 @@
         <v>215</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G74" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="I74" s="3" t="s">
         <v>29</v>
@@ -4742,12 +4752,12 @@
         <v>230</v>
       </c>
       <c r="L74" s="3" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>214</v>
@@ -4756,19 +4766,19 @@
         <v>215</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G75" s="3" t="s">
         <v>27</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="I75" s="3" t="s">
         <v>29</v>
@@ -4780,12 +4790,12 @@
         <v>230</v>
       </c>
       <c r="L75" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>376</v>
@@ -4794,22 +4804,22 @@
         <v>215</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J76" s="3" t="s">
         <v>21</v>
@@ -4818,12 +4828,12 @@
         <v>230</v>
       </c>
       <c r="L76" s="3" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>376</v>
@@ -4832,22 +4842,22 @@
         <v>215</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="I77" s="3" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="J77" s="3" t="s">
         <v>21</v>
@@ -4856,12 +4866,12 @@
         <v>230</v>
       </c>
       <c r="L77" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>376</v>
@@ -4870,22 +4880,22 @@
         <v>215</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="H78" s="3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="J78" s="3" t="s">
         <v>21</v>
@@ -4894,12 +4904,12 @@
         <v>230</v>
       </c>
       <c r="L78" s="3" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>75</v>
@@ -4908,36 +4918,36 @@
         <v>76</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="G79" s="3" t="s">
         <v>45</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="J79" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K79" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="L79" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>376</v>
@@ -4946,36 +4956,36 @@
         <v>215</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J80" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K80" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="L80" s="3" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>376</v>
@@ -4984,36 +4994,36 @@
         <v>215</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="I81" s="3" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J81" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="L81" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>376</v>
@@ -5022,31 +5032,31 @@
         <v>215</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="I82" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="J82" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K82" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="L82" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
   </sheetData>
@@ -5090,12 +5100,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5103,16 +5113,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>397</v>
+        <v>506</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5356,7 +5366,7 @@
       </c>
       <c r="C16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$100,$A16,'Test cases'!$J$2:$J$100,"Pass")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$100,$A16,'Test cases'!$J$2:$J$100,"Fail")</f>
@@ -5364,12 +5374,12 @@
       </c>
       <c r="E16" s="7" t="n">
         <f aca="false">COUNTIFS('Test cases'!$B$2:$B$100,$A16,'Test cases'!$J$2:$J$100,"Not run")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">SUM(B5:B16)</f>
@@ -5377,7 +5387,7 @@
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">SUM(C5:C16)</f>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D17" s="8" t="n">
         <f aca="false">SUM(D5:D16)</f>
@@ -5385,7 +5395,7 @@
       </c>
       <c r="E17" s="8" t="n">
         <f aca="false">SUM(E5:E16)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5397,7 +5407,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -5406,7 +5416,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"1")</f>
@@ -5421,7 +5431,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"2")</f>
@@ -5436,7 +5446,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"3")</f>
@@ -5451,7 +5461,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">COUNTIF('Test cases'!$C$2:$C$100,"4")</f>
@@ -5495,42 +5505,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>